<commit_message>
Add ZSWIM8-6 master grant template (all fund types) + 51 domain-specific corpus sentences (101 total) + full 6-part skeleton + eligibility self-check
</commit_message>
<xml_diff>
--- a/data/grant_writing_corpus.xlsx
+++ b/data/grant_writing_corpus.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +39,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +91,11 @@
         <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A148C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -114,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -167,6 +176,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -533,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2327,6 +2340,1804 @@
         </is>
       </c>
       <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr"/>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>🔬 领域专用句式（AMPK–TDMD / miRNA 方向）</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="inlineStr"/>
+      <c r="D52" s="19" t="inlineStr"/>
+      <c r="E52" s="19" t="inlineStr"/>
+      <c r="F52" s="19" t="inlineStr"/>
+      <c r="G52" s="19" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>开场钩子 Opening hook</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>MicroRNAs, once thought to be stable, are actively destroyed by target-directed miRNA decay (TDMD), in which the ZSWIM8 ubiquitin ligase marks target-engaged AGO2 for destruction.</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="inlineStr">
+        <is>
+          <t>TDMD 领域标准开场:一句把&amp;quot;miRNA 其实会被主动降解&amp;quot;这个反直觉点抛给评审。</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>NIH/优青/通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>开场钩子 Opening hook</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>紧迫 Urgency</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>Fibrosis is driven in part by loss of anti-fibrotic miR-29, yet what accelerates its turnover in diseased tissue remains unknown.</t>
+        </is>
+      </c>
+      <c r="F54" s="20" t="inlineStr">
+        <is>
+          <t>疾病导向紧迫开场,直接把 miR-29 与纤维化钉在一起(你的旗舰疾病轴)。</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>知识缺口 Knowledge gap</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>Although the ZSWIM8 TDMD machinery is now structurally defined, whether and how it is tuned by cellular metabolic state has not been tested.</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>把&amp;quot;结构已清楚、调控未知&amp;quot;做成缺口——你项目的核心留白。</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>NIH/优青/通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>知识缺口 Knowledge gap</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>TUT4/7-mediated uridylation controls pre-miRNA fate, but its coupling to sterol and lactate signaling in cancer has not been explored.</t>
+        </is>
+      </c>
+      <c r="F56" s="20" t="inlineStr">
+        <is>
+          <t>TUT4/7×胆固醇/乳酸方向的缺口句(你的第二候选轴)。</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>长期目标 Long-term goal</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Our long-term goal is to define the metabolic control of miRNA stability and to exploit it therapeutically in fibrosis and metabolic disease.</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="inlineStr">
+        <is>
+          <t>长期目标句:把&amp;quot;代谢控制 miRNA 稳定性&amp;quot;立成你实验室的招牌方向。</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>中心假设 Central hypothesis</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>Our central hypothesis is that AMPK phosphorylates ZSWIM8 at S608, accelerating TDMD of miR-29 and thereby encoding a metabolic memory of prior nutrient stress.</t>
+        </is>
+      </c>
+      <c r="F58" s="20" t="inlineStr">
+        <is>
+          <t>旗舰中心假设,一句含&amp;quot;激酶-底物-位点-miRNA-疾病记忆&amp;quot;完整链条。</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>中心假设 Central hypothesis</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>谨慎 Hedged</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>We hypothesize that nutrient stress, sensed by AMPK, shifts the rate of ZSWIM8-dependent miRNA decay, providing a tunable node linking metabolism to gene silencing.</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
+        <is>
+          <t>谨慎版中心假设(preliminary data 较弱时用 shift/tunable)。</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>NIH/通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Aim 拆分 Aim structure</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>Aim 1 will establish direct AMPK phosphorylation of ZSWIM8 at S608 in vitro; Aim 2 will define how this modification sets the rate of miR-29 TDMD; Aim 3 will test whether it encodes metabolic memory in fibrosis organoids.</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
+        <is>
+          <t>三 Aim 一句话总览:体外分子事件→功能读出→疾病记忆,逐级抬升。</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Aim 拆分 Aim structure</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>These aims are logically sequential yet independent: a negative result in Aim 3 would not invalidate the mechanistic advances of Aims 1–2.</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>评审最爱看的&amp;quot;层层递进但互不依赖&amp;quot;声明,降低风险印象。</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>收尾影响 Payoff</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>Successful completion will establish the first metabolic input to the TDMD machinery and define a phospho-switch (ZSWIM8-S608) as a druggable node in fibrosis.</t>
+        </is>
+      </c>
+      <c r="F62" s="20" t="inlineStr">
+        <is>
+          <t>收尾影响句:把成果拔高到&amp;quot;领域首个&amp;quot;+&amp;quot;可成药靶点&amp;quot;。</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>收尾影响 Payoff</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>By resolving how metabolism controls miRNA lifetime, this work opens a new axis for base-/prime-editing correction of fibrotic and dystrophic phenotypes.</t>
+        </is>
+      </c>
+      <c r="F63" s="20" t="inlineStr">
+        <is>
+          <t>把成果连到你的编辑技术长板(base/prime editing)。</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>NIH/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>可行性锚点 Feasibility anchor</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>Our motif scan places ZSWIM8-S608 in a textbook AMPK recognition context (…KRR-S608…) within a disordered, kinase-accessible region, providing a strong rationale for Aim 1.</t>
+        </is>
+      </c>
+      <c r="F64" s="20" t="inlineStr">
+        <is>
+          <t>把你自建 PSSM 打分的结果当可行性锚点(诚实标注 predicted)。</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>意义-临床 Clinical significance</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>紧迫 Urgency</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>Fibrosis contributes to nearly half of deaths in the developed world, yet no therapy restores the protective miR-29 program; a metabolic lever on its decay would be transformative.</t>
+        </is>
+      </c>
+      <c r="F65" s="20" t="inlineStr">
+        <is>
+          <t>临床分量句:大数字+现有疗法空白+你的切入点。</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>意义-机制 Mechanistic significance</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>Establishing AMPK as an upstream regulator of TDMD would convert miRNA turnover from a housekeeping process into a signal-responsive, druggable pathway.</t>
+        </is>
+      </c>
+      <c r="F66" s="20" t="inlineStr">
+        <is>
+          <t>机制意义:把&amp;quot;看家过程&amp;quot;重新定义为&amp;quot;可调可药&amp;quot;,提升想象空间。</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>意义-记忆 Metabolic memory</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>The concept of metabolic memory—persistent phenotypes after transient metabolic stress—remains molecularly unexplained; a durable ZSWIM8-S608 phospho-state offers a concrete mechanism.</t>
+        </is>
+      </c>
+      <c r="F67" s="20" t="inlineStr">
+        <is>
+          <t>把代谢记忆这个大概念落到你的分子机制上。</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>意义-通用性 Generality</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>Because ZSWIM8 governs decay of many miRNAs, a metabolic input would have broad consequences across the miRNAome, not just miR-29.</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>把单个 miRNA 的发现扩展到全 miRNAome 的普适意义。</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>NIH/通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>意义-代谢轴 Metabolic axis</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>Lactate and lactylation are emerging as signaling metabolites; linking them to TDMD would connect the Warburg-like state of fibrotic and tumor tissue to miRNA control.</t>
+        </is>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
+        <is>
+          <t>乳酸/乳酰化×TDMD 的意义句(你的代谢护城河)。</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>意义-胆固醇 Cholesterol axis</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>miR-33 sits at the intersection of cholesterol homeostasis and AMPK signaling; understanding its uridylation-dependent decay would inform both atherosclerosis and metabolic disease.</t>
+        </is>
+      </c>
+      <c r="F70" s="20" t="inlineStr">
+        <is>
+          <t>miR-33×胆固醇×AMPK 的意义句。</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>意义-疾病模型 Disease model</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E71" s="20" t="inlineStr">
+        <is>
+          <t>Our access to intestinal, cardiac, and dystrophic organoid models positions us to test metabolic control of miRNA decay directly in human-relevant tissue.</t>
+        </is>
+      </c>
+      <c r="F71" s="20" t="inlineStr">
+        <is>
+          <t>把你的类器官模型群当作独特资源写进意义。</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>NIH/NRF/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>意义-物种 Translational species</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>Findings will be validated in a T2D pig model, bridging the gap between rodent mechanism and large-animal translation.</t>
+        </is>
+      </c>
+      <c r="F72" s="20" t="inlineStr">
+        <is>
+          <t>T2D 猪模型的转化分量句(你的差异化资源)。</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>创新-概念 Conceptual</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>This work introduces a conceptual shift: miRNA decay is not constitutive but is set by the cell's metabolic state through a defined kinase–ligase axis.</t>
+        </is>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
+        <is>
+          <t>概念创新句:一句点明范式转变(constitutive→signal-set)。</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>创新-靶点 New target</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>We identify ZSWIM8-S608 as, to our knowledge, the first phosphosite proposed to couple energy sensing to target-directed miRNA decay.</t>
+        </is>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
+        <is>
+          <t>&amp;quot;首个&amp;quot;靶点声明(用 to our knowledge 保稳)。</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>创新-工具 Methodological</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E75" s="20" t="inlineStr">
+        <is>
+          <t>We combine a transparent, custom AMPK substrate-motif scorer with phospho-mimetic editing and single-miRNA decay kinetics—an integrated pipeline not previously applied to TDMD.</t>
+        </is>
+      </c>
+      <c r="F75" s="20" t="inlineStr">
+        <is>
+          <t>方法创新:把你的自建打分器+编辑+动力学串成新流水线。</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>NIH/NSF/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>创新-编辑 Editing</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>Rather than knockdown, we use base and prime editing to install precise S608A/S608D alleles at the endogenous locus, avoiding overexpression artifacts.</t>
+        </is>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>把 base/prime editing 当创新点(内源精确等位,避免过表达假象)。</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>创新-模型 Model system</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E77" s="20" t="inlineStr">
+        <is>
+          <t>Fibrosis organoids subjected to defined nutrient-stress pulses allow us to model metabolic memory with temporal control unattainable in vivo.</t>
+        </is>
+      </c>
+      <c r="F77" s="20" t="inlineStr">
+        <is>
+          <t>类器官+营养脉冲当作可控记忆模型的创新。</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>NIH/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>创新-跨领域 Cross-field</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E78" s="20" t="inlineStr">
+        <is>
+          <t>By uniting metabolism, RNA turnover, and ubiquitin signaling, this program occupies white space between fields that rarely intersect.</t>
+        </is>
+      </c>
+      <c r="F78" s="20" t="inlineStr">
+        <is>
+          <t>跨领域交叉创新句(诚实:强调交叉,不吹&amp;quot;全新&amp;quot;)。</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>创新-乳酰化 Lactylation</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E79" s="20" t="inlineStr">
+        <is>
+          <t>We test whether lactylation, a recently described modification, provides a parallel metabolic input to the TDMD machinery alongside AMPK phosphorylation.</t>
+        </is>
+      </c>
+      <c r="F79" s="20" t="inlineStr">
+        <is>
+          <t>把乳酰化作为&amp;quot;第二条代谢输入&amp;quot;的前瞻创新。</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>实验设计 Design</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E80" s="20" t="inlineStr">
+        <is>
+          <t>In vitro kinase assays with recombinant AMPK and ZSWIM8 fragments, phospho-specific detection, and S608A/S608D mutants will establish direct phosphorylation and its motif dependence.</t>
+        </is>
+      </c>
+      <c r="F80" s="20" t="inlineStr">
+        <is>
+          <t>Aim1 标准设计句:体外激酶+磷酸特异检测+点突变。</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>读出 Readout</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E81" s="20" t="inlineStr">
+        <is>
+          <t>miR-29 decay kinetics will be measured by time-resolved small-RNA sequencing after transcriptional shut-off in ZSWIM8-reconstituted cells.</t>
+        </is>
+      </c>
+      <c r="F81" s="20" t="inlineStr">
+        <is>
+          <t>衰减动力学读出句(转录关闭后测半衰期)。</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>定量 Quantification</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E82" s="20" t="inlineStr">
+        <is>
+          <t>Decay rate constants (k) will be fit per genotype; we expect S608D &gt; WT &gt; S608A &gt; ZSWIM8-KO, providing a quantitative test of the phospho-switch model.</t>
+        </is>
+      </c>
+      <c r="F82" s="20" t="inlineStr">
+        <is>
+          <t>把预期 k 排序写清楚(诚实标注 predicted),让评审看到可证伪。</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>备选方案 Alternative</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>谨慎 Hedged</t>
+        </is>
+      </c>
+      <c r="E83" s="20" t="inlineStr">
+        <is>
+          <t>Should S608 phosphorylation prove insufficient, we will test the neighboring S609 and S1202 sites, which our scan also flagged, and probe for AMPK-independent kinases.</t>
+        </is>
+      </c>
+      <c r="F83" s="20" t="inlineStr">
+        <is>
+          <t>备选方案句:预置 S609/S1202 备胎(你打分器排序里的现成候选)。</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>陷阱与对策 Pitfalls</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>谨慎 Hedged</t>
+        </is>
+      </c>
+      <c r="E84" s="20" t="inlineStr">
+        <is>
+          <t>A potential pitfall is that phospho-mimetic S608D may not fully recapitulate phosphorylation; we will corroborate with in-vitro-phosphorylated protein and phospho-specific antibodies.</t>
+        </is>
+      </c>
+      <c r="F84" s="20" t="inlineStr">
+        <is>
+          <t>主动写陷阱+对策,展示严谨性(评审加分项)。</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>模型系统 Model</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E85" s="20" t="inlineStr">
+        <is>
+          <t>Intestinal and cardiac fibrosis organoids will receive a defined nutrient-stress pulse, after which miR-29 levels and pro-fibrotic markers (SAA3, collagen) will be tracked for 7–14 days.</t>
+        </is>
+      </c>
+      <c r="F85" s="20" t="inlineStr">
+        <is>
+          <t>Aim3 类器官记忆实验设计(含 SAA3 等你的标志物)。</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>编辑策略 Editing strategy</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E86" s="20" t="inlineStr">
+        <is>
+          <t>Endogenous S608A and S608D alleles will be installed by prime editing; edited clones will be validated by amplicon sequencing before phenotyping.</t>
+        </is>
+      </c>
+      <c r="F86" s="20" t="inlineStr">
+        <is>
+          <t>prime editing 精确改位点的操作句。</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>体内验证 In vivo</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E87" s="20" t="inlineStr">
+        <is>
+          <t>Key findings will be confirmed in a bleomycin fibrosis model and, for translation, in a T2D pig model under controlled metabolic challenge.</t>
+        </is>
+      </c>
+      <c r="F87" s="20" t="inlineStr">
+        <is>
+          <t>体内+大动物验证句(bleomycin 经典纤维化 + 猪转化)。</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>统计与效力 Statistics</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E88" s="20" t="inlineStr">
+        <is>
+          <t>Group sizes were determined by power analysis to detect a 30% difference in decay rate at 80% power (α=0.05); all kinetic experiments use ≥3 biological replicates.</t>
+        </is>
+      </c>
+      <c r="F88" s="20" t="inlineStr">
+        <is>
+          <t>统计与样本量声明(NIH 严谨性硬要求)。</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>NIH/优青/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>严谨性-性别 SABV</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E89" s="20" t="inlineStr">
+        <is>
+          <t>Both sexes will be studied, and sex will be included as a biological variable in all animal and organoid experiments.</t>
+        </is>
+      </c>
+      <c r="F89" s="20" t="inlineStr">
+        <is>
+          <t>NIH 强制的 SABV 声明,直接可用。</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>NIH</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>严谨性-试剂 Rigor reagents</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E90" s="20" t="inlineStr">
+        <is>
+          <t>All antibodies, cell lines, and ZSWIM8 constructs will be authenticated (STR profiling, sequencing) and reported per RRID standards.</t>
+        </is>
+      </c>
+      <c r="F90" s="20" t="inlineStr">
+        <is>
+          <t>试剂鉴定与 RRID 声明,满足可重复性栏。</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>里程碑 Milestones</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E91" s="20" t="inlineStr">
+        <is>
+          <t>Go/no-go milestone: Aim 1 must confirm direct S608 phosphorylation before Aim 2 kinetics proceed, ensuring resources track validated mechanism.</t>
+        </is>
+      </c>
+      <c r="F91" s="20" t="inlineStr">
+        <is>
+          <t>go/no-go 里程碑句,体现项目管理(K99/R00 尤其看重)。</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>NIH/NRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>时间线 Timeline</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E92" s="20" t="inlineStr">
+        <is>
+          <t>Aim 1 (Yr 1–2, mentored K99 phase) builds the mechanistic foundation; Aims 2–3 (Yr 3–5, independent R00 phase) establish function and disease relevance.</t>
+        </is>
+      </c>
+      <c r="F92" s="20" t="inlineStr">
+        <is>
+          <t>把 Aim 与 K99→R00 阶段绑定的时间线句(K99 专用)。</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>NIH K99/R00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Candidate 职业发展</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>过渡逻辑 Transition</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E93" s="20" t="inlineStr">
+        <is>
+          <t>The mentored phase will provide advanced training in quantitative RNA-decay measurement and in vivo fibrosis modeling, skills I will carry into my independent program.</t>
+        </is>
+      </c>
+      <c r="F93" s="20" t="inlineStr">
+        <is>
+          <t>K99 段:把训练内容与独立后计划挂钩(mentored→independent)。</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>NIH K99/R00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Candidate 职业发展</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>独立性 Independence</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E94" s="20" t="inlineStr">
+        <is>
+          <t>The R00 phase establishes an independent research program on metabolic control of miRNA stability, distinct from my mentor's focus on TDMD structure.</t>
+        </is>
+      </c>
+      <c r="F94" s="20" t="inlineStr">
+        <is>
+          <t>R00 段:明确与导师课题划清界限,强调独立性。</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>NIH K99/R00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Candidate 职业发展</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>代表作 Track record</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E95" s="20" t="inlineStr">
+        <is>
+          <t>My seven first-author publications in RNA biology and metabolic disease establish my capacity to lead this interdisciplinary program.</t>
+        </is>
+      </c>
+      <c r="F95" s="20" t="inlineStr">
+        <is>
+          <t>海外优青/NRF 强调代表作:量化你的一作产出。</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>优青/NRF/RGC</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Candidate 职业发展</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>导师团队 Mentoring team</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E96" s="20" t="inlineStr">
+        <is>
+          <t>My mentoring team spans TDMD biochemistry, kinase signaling, and organoid disease modeling, covering every methodology in this proposal.</t>
+        </is>
+      </c>
+      <c r="F96" s="20" t="inlineStr">
+        <is>
+          <t>K99 导师团队覆盖度声明。</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>NIH K99/R00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Candidate 职业发展</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>国家需求 National need</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E97" s="20" t="inlineStr">
+        <is>
+          <t>Returning to establish an independent laboratory, I will address fibrosis and metabolic disease—major national health burdens—using the metabolic-miRNA axis.</t>
+        </is>
+      </c>
+      <c r="F97" s="20" t="inlineStr">
+        <is>
+          <t>海外优青:把课题连到国家需求(评审多为国内同行)。</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>连接词 Connectors</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>递进 Building</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E98" s="20" t="inlineStr">
+        <is>
+          <t>Building on our finding that S608 lies in an AMPK motif, we next asked whether phosphorylation alters ZSWIM8 activity toward miR-29.</t>
+        </is>
+      </c>
+      <c r="F98" s="20" t="inlineStr">
+        <is>
+          <t>&amp;quot;承上启下&amp;quot;连接句(从位点发现推进到功能)。</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>连接词 Connectors</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>对照 Contrast</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E99" s="20" t="inlineStr">
+        <is>
+          <t>In contrast to canonical miRNA biogenesis, which is transcriptionally set, TDMD offers a post-transcriptional, rapidly reversible control point.</t>
+        </is>
+      </c>
+      <c r="F99" s="20" t="inlineStr">
+        <is>
+          <t>对照连接句(把 TDMD 与经典生成通路对比)。</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>连接词 Connectors</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>因果 Causal</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>中性 Neutral</t>
+        </is>
+      </c>
+      <c r="E100" s="20" t="inlineStr">
+        <is>
+          <t>Because AMPK is activated within minutes of energy stress, any ZSWIM8 phospho-switch would allow miRNA levels to track metabolic state in near-real time.</t>
+        </is>
+      </c>
+      <c r="F100" s="20" t="inlineStr">
+        <is>
+          <t>因果连接句(把激酶动力学连到 miRNA 实时响应)。</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>语气 Tone</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>自信 Assertive</t>
+        </is>
+      </c>
+      <c r="E101" s="20" t="inlineStr">
+        <is>
+          <t>Our data demonstrate that ZSWIM8 depletion stabilizes miR-29, establishing TDMD as the dominant route of its turnover.</t>
+        </is>
+      </c>
+      <c r="F101" s="20" t="inlineStr">
+        <is>
+          <t>有数据时的自信定论句(demonstrate/establish)。</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>NIH/优青</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>语气 Tone</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>谨慎 Hedged</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>谨慎 Hedged</t>
+        </is>
+      </c>
+      <c r="E102" s="20" t="inlineStr">
+        <is>
+          <t>These results are consistent with, but do not yet prove, direct AMPK phosphorylation of ZSWIM8 in cells.</t>
+        </is>
+      </c>
+      <c r="F102" s="20" t="inlineStr">
+        <is>
+          <t>推断未定论时的谨慎句(consistent with/do not yet prove)。</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>NIH/通用</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>语气 Tone</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>紧迫 Urgency</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>紧迫 Urgency</t>
+        </is>
+      </c>
+      <c r="E103" s="20" t="inlineStr">
+        <is>
+          <t>With no approved therapy that restores anti-fibrotic miR-29, defining a metabolic lever on its decay is an urgent and tractable goal.</t>
+        </is>
+      </c>
+      <c r="F103" s="20" t="inlineStr">
+        <is>
+          <t>紧迫收束句(空白+可操作性并列)。</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
         <is>
           <t>NIH/优青</t>
         </is>
@@ -2356,12 +4167,8 @@
           <t>基金写作语料库 · Grant-Writing Sentence Bank</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>

</xml_diff>